<commit_message>
Add advanced differentiating features to the gap analysis document
Integrate the "Valore Aggiunto W3Suite" section into the gap analysis markdown and excel files, detailing AI Voice Agents, MCP Gateway, Universal Workflow Engine, and WebRTC Calls.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: bd83b791-fe19-4f8c-8f08-c40cf927c2eb
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: f75df62f-05c9-4bf5-b428-a2f48430e5f4
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/990d2e08-e877-47ab-86e4-4ab1ec4a5b18/bd83b791-fe19-4f8c-8f08-c40cf927c2eb/orRbN4m
</commit_message>
<xml_diff>
--- a/docs/gara-appalto/GAP-ANALYSIS-GESTIONALE-MIO-NEGOZIO.xlsx
+++ b/docs/gara-appalto/GAP-ANALYSIS-GESTIONALE-MIO-NEGOZIO.xlsx
@@ -5,6 +5,7 @@
   <sheets>
     <sheet name="Gap Analysis" sheetId="1" r:id="rId1"/>
     <sheet name="Gap Critici" sheetId="2" r:id="rId2"/>
+    <sheet name="Valore Aggiunto" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -399,16 +400,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:H67"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-    <col min="3" max="3" width="45.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="8.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="35.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1876,13 +1867,6 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E12"/>
-  <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" customWidth="1"/>
-    <col min="5" max="5" width="25.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2059,4 +2043,721 @@
     <ignoredError numberStoredAsText="1" sqref="A1:E12"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D64"/>
+  <cols>
+    <col min="1" max="1" width="5.83203125" customWidth="1"/>
+    <col min="2" max="2" width="40.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>VALORE AGGIUNTO W3SUITE - Capacità Distintive</v>
+      </c>
+      <c r="B1" t="str">
+        <v/>
+      </c>
+      <c r="C1" t="str">
+        <v/>
+      </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>#</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Funzionalità</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Tecnologia</v>
+      </c>
+      <c r="D3" t="str">
+        <v>Benefici WindTre</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>1</v>
+      </c>
+      <c r="B5" t="str">
+        <v>AGENTI AI RAGGIUNGIBILI</v>
+      </c>
+      <c r="C5" t="str">
+        <v>AI Voice Agent + RAG</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v/>
+      </c>
+      <c r="B6" t="str">
+        <v>- Assistente vocale AI 24/7</v>
+      </c>
+      <c r="C6" t="str">
+        <v>OpenAI GPT-4 + RAG</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Riduzione carico call center 40-60%</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v>- Context-aware (cliente, ordini, storico)</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Knowledge Base dinamica</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Risposta immediata h24</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+      <c r="B8" t="str">
+        <v>- Handoff automatico a operatore umano</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Intelligent Routing</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Standardizzazione qualità supporto</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+      <c r="B9" t="str">
+        <v>- Multi-lingua italiano/inglese</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>2</v>
+      </c>
+      <c r="B11" t="str">
+        <v>MCP GATEWAY</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Multi-Channel Provider Gateway</v>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v/>
+      </c>
+      <c r="B12" t="str">
+        <v>- Single Point of Integration</v>
+      </c>
+      <c r="C12" t="str">
+        <v>API Gateway unificato</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Integrazione semplificata sistemi WindTre</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v/>
+      </c>
+      <c r="B13" t="str">
+        <v>- Provider: OpenAI, Twilio, WhatsApp, SMS</v>
+      </c>
+      <c r="C13" t="str">
+        <v>OAuth2/OIDC</v>
+      </c>
+      <c r="D13" t="str">
+        <v>Riduzione tempi sviluppo 70%</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v/>
+      </c>
+      <c r="B14" t="str">
+        <v>- Fallback automatico tra provider</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Rate Limiting granulare</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Governance centralizzata accessi API</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v/>
+      </c>
+      <c r="B15" t="str">
+        <v>- Audit completo tutte interazioni</v>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>3</v>
+      </c>
+      <c r="B17" t="str">
+        <v>UNIVERSAL WORKFLOW ENGINE</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Visual Builder + AI</v>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v/>
+      </c>
+      <c r="B18" t="str">
+        <v>- Drag-and-drop senza codice</v>
+      </c>
+      <c r="C18" t="str">
+        <v>AI Workflow Builder</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Time-to-market: settimane → ore</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v/>
+      </c>
+      <c r="B19" t="str">
+        <v>- Intelligent Routing (regole, turni, competenze)</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Trigger multipli</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Standardizzazione processi rete</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v/>
+      </c>
+      <c r="B20" t="str">
+        <v>- Cross-store workflows</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Template library</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Adattabilità rapida nuove esigenze</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v/>
+      </c>
+      <c r="B21" t="str">
+        <v>- Versioning con rollback</v>
+      </c>
+      <c r="C21" t="str">
+        <v/>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>4</v>
+      </c>
+      <c r="B23" t="str">
+        <v>SISTEMA CHIAMATE WebRTC</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Browser-based real-time</v>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v/>
+      </c>
+      <c r="B24" t="str">
+        <v>- Click-to-call dal CRM</v>
+      </c>
+      <c r="C24" t="str">
+        <v>WebRTC + SIP</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Eliminazione costi licenze softphone</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v/>
+      </c>
+      <c r="B25" t="str">
+        <v>- Softphone integrato nel browser</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Recording + Trascrizione AI</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Integrazione nativa CRM</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v/>
+      </c>
+      <c r="B26" t="str">
+        <v>- Whisper mode / Barge-in supervisor</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Video call + Screen sharing</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Analytics chiamate</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v/>
+      </c>
+      <c r="B27" t="str">
+        <v>- IVR dinamico configurabile</v>
+      </c>
+      <c r="C27" t="str">
+        <v/>
+      </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>5</v>
+      </c>
+      <c r="B29" t="str">
+        <v>AI ENFORCEMENT MIDDLEWARE</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Quality Assurance Layer</v>
+      </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v/>
+      </c>
+      <c r="B30" t="str">
+        <v>- Content moderation automatica</v>
+      </c>
+      <c r="C30" t="str">
+        <v>AI Policy Enforcement</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Riduzione rischio compliance</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v/>
+      </c>
+      <c r="B31" t="str">
+        <v>- Compliance check AGCOM/privacy</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Quality scoring real-time</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Miglioramento qualità +15%</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v/>
+      </c>
+      <c r="B32" t="str">
+        <v>- Anomaly detection frodi</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Suggestion engine</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Early warning problematiche</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>6</v>
+      </c>
+      <c r="B34" t="str">
+        <v>ANALYTICS AI-POWERED</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Predictive BI</v>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v/>
+      </c>
+      <c r="B35" t="str">
+        <v>- Predictive analytics (vendite, churn)</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Natural language queries</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Decision-making data-driven</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v/>
+      </c>
+      <c r="B36" t="str">
+        <v>- Automated insights con trend</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Benchmark automatico</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Riduzione tempo analisi 80%</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v/>
+      </c>
+      <c r="B37" t="str">
+        <v>- What-if analysis scenari</v>
+      </c>
+      <c r="C37" t="str">
+        <v/>
+      </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>7</v>
+      </c>
+      <c r="B39" t="str">
+        <v>ARCHITETTURA ENTERPRISE-GRADE</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Security &amp; Compliance</v>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v/>
+      </c>
+      <c r="B40" t="str">
+        <v>- Multi-tenant nativo</v>
+      </c>
+      <c r="C40" t="str">
+        <v>PostgreSQL RLS</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Isolamento completo dealer</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v/>
+      </c>
+      <c r="B41" t="str">
+        <v>- 3-level RBAC</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Zero-trust</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Controllo accessi granulare</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v/>
+      </c>
+      <c r="B42" t="str">
+        <v>- Audit immutabile (event sourcing)</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Encryption AES-256/TLS 1.3</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Tracciabilità completa</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>CONFRONTO COMPETITIVO</v>
+      </c>
+      <c r="B45" t="str">
+        <v/>
+      </c>
+      <c r="C45" t="str">
+        <v/>
+      </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Funzionalità</v>
+      </c>
+      <c r="B47" t="str">
+        <v>W3Suite</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Competitor A</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Competitor B</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>AI Voice Agent</v>
+      </c>
+      <c r="B48" t="str">
+        <v>NATIVO</v>
+      </c>
+      <c r="C48" t="str">
+        <v>NO</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Add-on</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>MCP Gateway</v>
+      </c>
+      <c r="B49" t="str">
+        <v>NATIVO</v>
+      </c>
+      <c r="C49" t="str">
+        <v>NO</v>
+      </c>
+      <c r="D49" t="str">
+        <v>NO</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Workflow AI Builder</v>
+      </c>
+      <c r="B50" t="str">
+        <v>NATIVO</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Basic</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Basic</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>WebRTC Calls</v>
+      </c>
+      <c r="B51" t="str">
+        <v>NATIVO</v>
+      </c>
+      <c r="C51" t="str">
+        <v>NO</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Add-on</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>AI Enforcement</v>
+      </c>
+      <c r="B52" t="str">
+        <v>NATIVO</v>
+      </c>
+      <c r="C52" t="str">
+        <v>NO</v>
+      </c>
+      <c r="D52" t="str">
+        <v>NO</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Predictive Analytics</v>
+      </c>
+      <c r="B53" t="str">
+        <v>NATIVO</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Basic</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Basic</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Multi-tenant RLS</v>
+      </c>
+      <c r="B54" t="str">
+        <v>NATIVO</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Parziale</v>
+      </c>
+      <c r="D54" t="str">
+        <v>NO</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>ROI STIMATO VALORE AGGIUNTO</v>
+      </c>
+      <c r="B57" t="str">
+        <v/>
+      </c>
+      <c r="C57" t="str">
+        <v/>
+      </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Funzionalità</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Risparmio/Beneficio Annuo</v>
+      </c>
+      <c r="C59" t="str">
+        <v/>
+      </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>AI Voice Agent 24/7</v>
+      </c>
+      <c r="B60" t="str">
+        <v>-40% costi call center</v>
+      </c>
+      <c r="C60" t="str">
+        <v/>
+      </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>Workflow automation</v>
+      </c>
+      <c r="B61" t="str">
+        <v>-60% tempo gestione processi</v>
+      </c>
+      <c r="C61" t="str">
+        <v/>
+      </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>WebRTC integrato</v>
+      </c>
+      <c r="B62" t="str">
+        <v>-100% licenze softphone</v>
+      </c>
+      <c r="C62" t="str">
+        <v/>
+      </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>AI Quality scoring</v>
+      </c>
+      <c r="B63" t="str">
+        <v>+15% customer satisfaction</v>
+      </c>
+      <c r="C63" t="str">
+        <v/>
+      </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>Predictive analytics</v>
+      </c>
+      <c r="B64" t="str">
+        <v>+10% vendite (ottimizzazione stock)</v>
+      </c>
+      <c r="C64" t="str">
+        <v/>
+      </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:D64"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>